<commit_message>
Update the dashboard for week 5
- Plan follows the Gantt workbook revised on 2026-10-14: 25 tasks,
  WP3.1 renamed Detection, WP3.2-3.3 one week longer, WP5 split into
  five tasks; the workbook snapshot is replaced.
- Tasks carry status, percent progress and team members; package
  headers show the mean progress. WP6 reflects the VoltEPIC site.
- Week 5 review record and the first latest-update entry.
- Sidebar link to the analysis website (VoltEPIC).
- Results & resources becomes three full-width tabs: Experiments &
  results, Library and Measurement campaign.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/PeakDeconv_Gantt_Chart.xlsx
+++ b/documents/PeakDeconv_Gantt_Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Voltammetry\plan\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Voltammetry\ENG\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_EA0542486DC139E9FCD199BFDB7E6980C92352A0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{682827E3-EEB1-4B02-A828-2F19DF72D70D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4590" yWindow="2190" windowWidth="38700" windowHeight="17745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt chart" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,17 @@
     <sheet name="Task overview" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Gantt chart'!$A$1:$Q$55</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Task overview'!$A$1:$E$33</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Team 1 · DL'!$A$1:$Q$55</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Team 2 · ML'!$A$1:$Q$55</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Gantt chart'!$A$1:$Q$57</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Task overview'!$A$1:$E$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Team 1 · DL'!$A$1:$Q$57</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Team 2 · ML'!$A$1:$Q$57</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="146">
   <si>
     <t>Project work plan</t>
   </si>
@@ -151,7 +151,7 @@
     <t>WP3.1</t>
   </si>
   <si>
-    <t>Analyte presence detection</t>
+    <t>Detection</t>
   </si>
   <si>
     <t>T1 DL | T2 ML</t>
@@ -220,19 +220,31 @@
     <t>WP5.1</t>
   </si>
   <si>
-    <t>XAI method selection and setup</t>
+    <t>Detection XAI — setup, explanations and reliability tests</t>
   </si>
   <si>
     <t>WP5.2</t>
   </si>
   <si>
-    <t>Explanation runs on project models</t>
+    <t>Classification XAI — explanations and reliability tests</t>
   </si>
   <si>
     <t>WP5.3</t>
   </si>
   <si>
-    <t>Explanation faithfulness and stability testing</t>
+    <t>Regression XAI — explanations and reliability tests</t>
+  </si>
+  <si>
+    <t>WP5.4</t>
+  </si>
+  <si>
+    <t>Local-data XAI — explanations and reliability tests</t>
+  </si>
+  <si>
+    <t>WP5.5</t>
+  </si>
+  <si>
+    <t>Cross-task comparison of explanations</t>
   </si>
   <si>
     <t>WP6</t>
@@ -301,169 +313,34 @@
     <t>Packages</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF009289"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP1 · Acquisition</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF772F6F"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP4 · Adaptation</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FFBB565A"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP6 · Interface</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF00578C"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP2 · Preprocessing</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF946200"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP5 · XAI</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF726DC4"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>WP3 · Models</t>
-    </r>
+    <t>■ WP1 · Acquisition</t>
+  </si>
+  <si>
+    <t>■ WP4 · Adaptation</t>
+  </si>
+  <si>
+    <t>■ WP6 · Interface</t>
+  </si>
+  <si>
+    <t>■ WP2 · Preprocessing</t>
+  </si>
+  <si>
+    <t>■ WP5 · XAI</t>
+  </si>
+  <si>
+    <t>■ WP3 · Models</t>
   </si>
   <si>
     <t>Owners</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF34495E"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">■ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>BME lead</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF9AA9B8"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">▣ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>EEE lead</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF34495E"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">▨ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color rgb="FF4B5560"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>BME + EEE</t>
-    </r>
+    <t>■ BME lead</t>
+  </si>
+  <si>
+    <t>▣ EEE lead</t>
+  </si>
+  <si>
+    <t>▨ BME + EEE</t>
   </si>
   <si>
     <t>Delivery</t>
@@ -538,60 +415,47 @@
     <t>WP3 · Model Development and Evaluation</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="8"/>
-        <color rgb="FF34495E"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t xml:space="preserve">EEE lead
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color rgb="FF34495E"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Team 1 · DL  |  Team 2 · ML</t>
-    </r>
-  </si>
-  <si>
-    <t>Weeks 4–5</t>
+    <t>EEE lead
+Team 1 · DL  |  Team 2 · ML</t>
+  </si>
+  <si>
+    <t>Weeks 4–6</t>
+  </si>
+  <si>
+    <t>Weeks 5–7</t>
+  </si>
+  <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>WP4 · Model Adaptation and Evaluation on Local Data</t>
+  </si>
+  <si>
+    <t>Weeks 6–7</t>
+  </si>
+  <si>
+    <t>Weeks 9–10</t>
+  </si>
+  <si>
+    <t>Weeks 9–11</t>
+  </si>
+  <si>
+    <t>Weeks 10–11</t>
+  </si>
+  <si>
+    <t>Weeks 12–14</t>
+  </si>
+  <si>
+    <t>WP5 · Explainable AI (XAI)</t>
+  </si>
+  <si>
+    <t>Weeks 3–4</t>
   </si>
   <si>
     <t>Weeks 5–6</t>
   </si>
   <si>
-    <t>Week 7</t>
-  </si>
-  <si>
-    <t>WP4 · Model Adaptation and Evaluation on Local Data</t>
-  </si>
-  <si>
-    <t>Weeks 6–7</t>
-  </si>
-  <si>
-    <t>Weeks 9–10</t>
-  </si>
-  <si>
-    <t>Weeks 9–11</t>
-  </si>
-  <si>
-    <t>Weeks 10–11</t>
-  </si>
-  <si>
-    <t>Weeks 12–14</t>
-  </si>
-  <si>
-    <t>WP5 · Explainable AI (XAI)</t>
-  </si>
-  <si>
-    <t>Weeks 3–7</t>
-  </si>
-  <si>
-    <t>Weeks 5–7, Weeks 9–12</t>
+    <t>Weeks 10–12</t>
   </si>
   <si>
     <t>Weeks 13–15</t>
@@ -613,7 +477,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0&quot; wk&quot;"/>
   </numFmts>
-  <fonts count="53" x14ac:knownFonts="1">
+  <fonts count="44" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -875,51 +739,6 @@
       <color rgb="FF4B5560"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF726DC4"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FFBB565A"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF009289"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF772F6F"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF00578C"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF946200"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF34495E"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF9AA9B8"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="7"/>
-      <color rgb="FF34495E"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
   <fills count="23">
     <fill>
@@ -1054,7 +873,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="139">
+  <borders count="140">
     <border>
       <left/>
       <right/>
@@ -2712,11 +2531,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD5D1C7"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF946200"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFEEECE6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="127"/>
   </cellStyleXfs>
-  <cellXfs count="200">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -3100,48 +2932,49 @@
     <xf numFmtId="0" fontId="15" fillId="22" borderId="137" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="139" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="127" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="127" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="90" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="126" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="93" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="95" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="67" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="126" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="96" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="92" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -3153,10 +2986,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="39" fillId="20" borderId="121" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="122" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="22" fillId="11" borderId="103" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -3177,6 +3006,10 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="109" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="121" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="122" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3482,7 +3315,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -3491,21 +3324,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O1" s="165" t="s">
+      <c r="O1" s="166" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
+      <c r="P1" s="167"/>
+      <c r="Q1" s="167"/>
     </row>
     <row r="2" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="185" t="s">
+      <c r="O2" s="186" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="166"/>
-      <c r="Q2" s="166"/>
+      <c r="P2" s="167"/>
+      <c r="Q2" s="167"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -3538,39 +3371,39 @@
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="171" t="s">
+      <c r="A7" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="172"/>
-      <c r="C7" s="177" t="s">
+      <c r="B7" s="169"/>
+      <c r="C7" s="178" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="172"/>
-      <c r="E7" s="172"/>
-      <c r="F7" s="172"/>
-      <c r="G7" s="177" t="s">
+      <c r="D7" s="169"/>
+      <c r="E7" s="169"/>
+      <c r="F7" s="169"/>
+      <c r="G7" s="178" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="172"/>
-      <c r="I7" s="172"/>
-      <c r="J7" s="172"/>
-      <c r="K7" s="177" t="s">
+      <c r="H7" s="169"/>
+      <c r="I7" s="169"/>
+      <c r="J7" s="169"/>
+      <c r="K7" s="178" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="172"/>
-      <c r="M7" s="172"/>
-      <c r="N7" s="172"/>
-      <c r="O7" s="179" t="s">
+      <c r="L7" s="169"/>
+      <c r="M7" s="169"/>
+      <c r="N7" s="169"/>
+      <c r="O7" s="180" t="s">
         <v>9</v>
       </c>
-      <c r="P7" s="172"/>
-      <c r="Q7" s="180"/>
+      <c r="P7" s="169"/>
+      <c r="Q7" s="181"/>
     </row>
     <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="173" t="s">
+      <c r="A8" s="164" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="178" t="s">
+      <c r="B8" s="179" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="5">
@@ -3620,8 +3453,8 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="174"/>
-      <c r="B9" s="166"/>
+      <c r="A9" s="165"/>
+      <c r="B9" s="167"/>
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
@@ -4009,10 +3842,12 @@
       <c r="F22" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="H22" s="19"/>
+      <c r="G22" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="I22" s="19"/>
       <c r="J22" s="21"/>
       <c r="K22" s="20"/>
@@ -4032,10 +3867,12 @@
       <c r="F23" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="G23" s="153" t="s">
+      <c r="G23" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="H23" s="19"/>
+      <c r="H23" s="153" t="s">
+        <v>41</v>
+      </c>
       <c r="I23" s="19"/>
       <c r="J23" s="21"/>
       <c r="K23" s="20"/>
@@ -4060,10 +3897,12 @@
       <c r="G24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="I24" s="19"/>
+      <c r="H24" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="J24" s="21"/>
       <c r="K24" s="20"/>
       <c r="L24" s="19"/>
@@ -4083,10 +3922,12 @@
       <c r="G25" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="H25" s="153" t="s">
+      <c r="H25" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="I25" s="19"/>
+      <c r="I25" s="153" t="s">
+        <v>41</v>
+      </c>
       <c r="J25" s="21"/>
       <c r="K25" s="20"/>
       <c r="L25" s="19"/>
@@ -4371,7 +4212,7 @@
       <c r="H36" s="91"/>
       <c r="I36" s="91"/>
       <c r="J36" s="17"/>
-      <c r="K36" s="92"/>
+      <c r="K36" s="163"/>
       <c r="L36" s="91"/>
       <c r="M36" s="91"/>
       <c r="N36" s="91"/>
@@ -4393,18 +4234,12 @@
       <c r="E37" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I37" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="F37" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="G37" s="20"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
       <c r="J37" s="21"/>
       <c r="K37" s="20"/>
       <c r="L37" s="19"/>
@@ -4428,25 +4263,15 @@
       <c r="G38" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I38" s="23" t="s">
-        <v>34</v>
-      </c>
+      <c r="H38" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" s="19"/>
       <c r="J38" s="21"/>
-      <c r="K38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N38" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="K38" s="20"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+      <c r="N38" s="19"/>
       <c r="O38" s="20"/>
       <c r="P38" s="19"/>
       <c r="Q38" s="22"/>
@@ -4463,65 +4288,61 @@
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="20"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
+      <c r="H39" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="151" t="s">
+        <v>34</v>
+      </c>
       <c r="J39" s="21"/>
       <c r="K39" s="20"/>
       <c r="L39" s="19"/>
       <c r="M39" s="19"/>
       <c r="N39" s="19"/>
-      <c r="O39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="P39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q39" s="150" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="96" t="s">
+      <c r="O39" s="20"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="22"/>
+    </row>
+    <row r="40" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="94" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="97" t="s">
+      <c r="B40" s="95" t="s">
         <v>69</v>
       </c>
-      <c r="C40" s="158"/>
-      <c r="D40" s="98"/>
-      <c r="E40" s="98"/>
-      <c r="F40" s="98"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="98"/>
-      <c r="I40" s="98"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="99"/>
-      <c r="L40" s="98"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="98"/>
-      <c r="O40" s="99"/>
-      <c r="P40" s="98"/>
-      <c r="Q40" s="100" t="s">
-        <v>17</v>
-      </c>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N40" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O40" s="20"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="22"/>
     </row>
     <row r="41" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="101" t="s">
+      <c r="A41" s="94" t="s">
         <v>70</v>
       </c>
-      <c r="B41" s="102" t="s">
+      <c r="B41" s="95" t="s">
         <v>71</v>
       </c>
       <c r="C41" s="19"/>
-      <c r="D41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="159" t="s">
-        <v>20</v>
-      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
       <c r="G41" s="20"/>
       <c r="H41" s="19"/>
       <c r="I41" s="19"/>
@@ -4530,48 +4351,40 @@
       <c r="L41" s="19"/>
       <c r="M41" s="19"/>
       <c r="N41" s="19"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="19"/>
-      <c r="Q41" s="22"/>
-    </row>
-    <row r="42" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="101" t="s">
+      <c r="O41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="P41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q41" s="150" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="96" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="102" t="s">
+      <c r="B42" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="J42" s="21"/>
-      <c r="K42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N42" s="151" t="s">
-        <v>34</v>
-      </c>
-      <c r="O42" s="20"/>
-      <c r="P42" s="19"/>
-      <c r="Q42" s="22"/>
+      <c r="C42" s="158"/>
+      <c r="D42" s="98"/>
+      <c r="E42" s="98"/>
+      <c r="F42" s="98"/>
+      <c r="G42" s="99"/>
+      <c r="H42" s="98"/>
+      <c r="I42" s="98"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="99"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="98"/>
+      <c r="O42" s="99"/>
+      <c r="P42" s="98"/>
+      <c r="Q42" s="100" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="43" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="101" t="s">
@@ -4581,188 +4394,256 @@
         <v>75</v>
       </c>
       <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
+      <c r="D43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="159" t="s">
+        <v>20</v>
+      </c>
       <c r="G43" s="20"/>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
       <c r="J43" s="21"/>
       <c r="K43" s="20"/>
       <c r="L43" s="19"/>
-      <c r="M43" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N43" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
       <c r="O43" s="20"/>
       <c r="P43" s="19"/>
       <c r="Q43" s="22"/>
     </row>
     <row r="44" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="103" t="s">
+      <c r="A44" s="101" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="104" t="s">
+      <c r="B44" s="102" t="s">
         <v>77</v>
       </c>
-      <c r="C44" s="105"/>
-      <c r="D44" s="105"/>
-      <c r="E44" s="105"/>
-      <c r="F44" s="105"/>
-      <c r="G44" s="106"/>
-      <c r="H44" s="105"/>
-      <c r="I44" s="105"/>
-      <c r="J44" s="107"/>
-      <c r="K44" s="106"/>
-      <c r="L44" s="105"/>
-      <c r="M44" s="105"/>
-      <c r="N44" s="105"/>
-      <c r="O44" s="108" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="J44" s="21"/>
+      <c r="K44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="L44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N44" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O44" s="20"/>
+      <c r="P44" s="19"/>
+      <c r="Q44" s="22"/>
+    </row>
+    <row r="45" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="101" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="102" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="19"/>
+      <c r="I45" s="19"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N45" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O45" s="20"/>
+      <c r="P45" s="19"/>
+      <c r="Q45" s="22"/>
+    </row>
+    <row r="46" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="103" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="106"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="107"/>
+      <c r="K46" s="106"/>
+      <c r="L46" s="105"/>
+      <c r="M46" s="105"/>
+      <c r="N46" s="105"/>
+      <c r="O46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="P44" s="108" t="s">
+      <c r="P46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="150" t="s">
+      <c r="Q46" s="150" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="186" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="187"/>
-      <c r="C45" s="187"/>
-      <c r="D45" s="187"/>
-      <c r="E45" s="187"/>
-      <c r="F45" s="187"/>
-      <c r="G45" s="187"/>
-      <c r="H45" s="187"/>
-      <c r="I45" s="187"/>
-      <c r="J45" s="187"/>
-      <c r="K45" s="187"/>
-      <c r="L45" s="187"/>
-      <c r="M45" s="187"/>
-      <c r="N45" s="187"/>
-      <c r="O45" s="187"/>
-      <c r="P45" s="187"/>
-      <c r="Q45" s="187"/>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C46" s="109" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="110" t="s">
-        <v>80</v>
-      </c>
-      <c r="D47" s="163" t="s">
-        <v>81</v>
-      </c>
-      <c r="E47" s="164"/>
-      <c r="F47" s="167" t="s">
+    <row r="47" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="187" t="s">
         <v>82</v>
       </c>
-      <c r="G47" s="168"/>
-    </row>
-    <row r="48" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="111" t="s">
+      <c r="B47" s="188"/>
+      <c r="C47" s="188"/>
+      <c r="D47" s="188"/>
+      <c r="E47" s="188"/>
+      <c r="F47" s="188"/>
+      <c r="G47" s="188"/>
+      <c r="H47" s="188"/>
+      <c r="I47" s="188"/>
+      <c r="J47" s="188"/>
+      <c r="K47" s="188"/>
+      <c r="L47" s="188"/>
+      <c r="M47" s="188"/>
+      <c r="N47" s="188"/>
+      <c r="O47" s="188"/>
+      <c r="P47" s="188"/>
+      <c r="Q47" s="188"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C48" s="109" t="s">
         <v>83</v>
       </c>
-      <c r="D48" s="183" t="s">
+    </row>
+    <row r="49" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="110" t="s">
         <v>84</v>
       </c>
-      <c r="E48" s="184"/>
-      <c r="F48" s="169" t="s">
+      <c r="D49" s="170" t="s">
         <v>85</v>
       </c>
-      <c r="G48" s="170"/>
-    </row>
-    <row r="49" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="112" t="s">
+      <c r="E49" s="171"/>
+      <c r="F49" s="176" t="s">
         <v>86</v>
       </c>
-      <c r="D49" s="175" t="s">
+      <c r="G49" s="177"/>
+    </row>
+    <row r="50" spans="3:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="E49" s="176"/>
-      <c r="F49" s="181" t="s">
+      <c r="D50" s="184" t="s">
         <v>88</v>
       </c>
-      <c r="G49" s="182"/>
+      <c r="E50" s="185"/>
+      <c r="F50" s="182" t="s">
+        <v>89</v>
+      </c>
+      <c r="G50" s="183"/>
     </row>
     <row r="51" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="113" t="s">
-        <v>89</v>
-      </c>
-      <c r="D51" s="114" t="s">
+      <c r="C51" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="F51" s="114" t="s">
+      <c r="D51" s="174" t="s">
         <v>91</v>
       </c>
-      <c r="H51" s="114" t="s">
+      <c r="E51" s="175"/>
+      <c r="F51" s="172" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="52" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D52" s="114" t="s">
+      <c r="G51" s="173"/>
+    </row>
+    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="113" t="s">
         <v>93</v>
       </c>
-      <c r="F52" s="114" t="s">
+      <c r="D53" s="114" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D53" s="114" t="s">
+      <c r="F53" s="114" t="s">
         <v>95</v>
       </c>
-      <c r="F53" s="114"/>
+      <c r="H53" s="114" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="54" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="113" t="s">
-        <v>96</v>
-      </c>
       <c r="D54" s="114" t="s">
         <v>97</v>
       </c>
-      <c r="E54" s="114" t="s">
+      <c r="F54" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="F54" s="114" t="s">
+    </row>
+    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D55" s="114" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="113" t="s">
+      <c r="F55" s="114"/>
+    </row>
+    <row r="56" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="113" t="s">
         <v>100</v>
       </c>
-      <c r="D55" s="151"/>
-      <c r="E55" s="149" t="s">
+      <c r="D56" s="114" t="s">
         <v>101</v>
+      </c>
+      <c r="E56" s="114" t="s">
+        <v>102</v>
+      </c>
+      <c r="F56" s="114" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="113" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" s="151"/>
+      <c r="E57" s="149" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="O1:Q1"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="D49:E49"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="F49:G49"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="O7:Q7"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="K7:N7"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="A45:Q45"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="O1:Q1"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="D50:E50"/>
     <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="A47:Q47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>
@@ -4774,7 +4655,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -4783,25 +4664,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O1" s="165" t="s">
+      <c r="O1" s="166" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
+      <c r="P1" s="167"/>
+      <c r="Q1" s="167"/>
     </row>
     <row r="2" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="185" t="s">
+      <c r="O2" s="186" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="166"/>
-      <c r="Q2" s="166"/>
+      <c r="P2" s="167"/>
+      <c r="Q2" s="167"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -4826,43 +4707,43 @@
     <row r="5" spans="1:17" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="171" t="s">
+      <c r="A7" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="172"/>
-      <c r="C7" s="177" t="s">
+      <c r="B7" s="169"/>
+      <c r="C7" s="178" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="172"/>
-      <c r="E7" s="172"/>
-      <c r="F7" s="172"/>
-      <c r="G7" s="177" t="s">
+      <c r="D7" s="169"/>
+      <c r="E7" s="169"/>
+      <c r="F7" s="169"/>
+      <c r="G7" s="178" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="172"/>
-      <c r="I7" s="172"/>
-      <c r="J7" s="172"/>
-      <c r="K7" s="177" t="s">
+      <c r="H7" s="169"/>
+      <c r="I7" s="169"/>
+      <c r="J7" s="169"/>
+      <c r="K7" s="178" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="172"/>
-      <c r="M7" s="172"/>
-      <c r="N7" s="172"/>
-      <c r="O7" s="179" t="s">
+      <c r="L7" s="169"/>
+      <c r="M7" s="169"/>
+      <c r="N7" s="169"/>
+      <c r="O7" s="180" t="s">
         <v>9</v>
       </c>
-      <c r="P7" s="172"/>
-      <c r="Q7" s="180"/>
+      <c r="P7" s="169"/>
+      <c r="Q7" s="181"/>
     </row>
     <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="173" t="s">
+      <c r="A8" s="164" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="178" t="s">
+      <c r="B8" s="179" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="5">
@@ -4912,8 +4793,8 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="174"/>
-      <c r="B9" s="166"/>
+      <c r="A9" s="165"/>
+      <c r="B9" s="167"/>
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
@@ -5268,13 +5149,13 @@
       <c r="B21" s="63"/>
       <c r="C21" s="19"/>
       <c r="D21" s="64" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E21" s="64" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="F21" s="153" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="G21" s="20"/>
       <c r="H21" s="19"/>
@@ -5301,10 +5182,12 @@
       <c r="F22" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="H22" s="19"/>
+      <c r="G22" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="I22" s="19"/>
       <c r="J22" s="21"/>
       <c r="K22" s="20"/>
@@ -5322,12 +5205,14 @@
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="64" t="s">
-        <v>104</v>
-      </c>
-      <c r="G23" s="153" t="s">
-        <v>104</v>
-      </c>
-      <c r="H23" s="19"/>
+        <v>108</v>
+      </c>
+      <c r="G23" s="64" t="s">
+        <v>108</v>
+      </c>
+      <c r="H23" s="153" t="s">
+        <v>108</v>
+      </c>
       <c r="I23" s="19"/>
       <c r="J23" s="21"/>
       <c r="K23" s="20"/>
@@ -5352,10 +5237,12 @@
       <c r="G24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="I24" s="19"/>
+      <c r="H24" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="J24" s="21"/>
       <c r="K24" s="20"/>
       <c r="L24" s="19"/>
@@ -5373,12 +5260,14 @@
       <c r="E25" s="19"/>
       <c r="F25" s="19"/>
       <c r="G25" s="65" t="s">
-        <v>104</v>
-      </c>
-      <c r="H25" s="153" t="s">
-        <v>104</v>
-      </c>
-      <c r="I25" s="19"/>
+        <v>108</v>
+      </c>
+      <c r="H25" s="65" t="s">
+        <v>108</v>
+      </c>
+      <c r="I25" s="153" t="s">
+        <v>108</v>
+      </c>
       <c r="J25" s="21"/>
       <c r="K25" s="20"/>
       <c r="L25" s="19"/>
@@ -5504,10 +5393,10 @@
       <c r="I30" s="19"/>
       <c r="J30" s="21"/>
       <c r="K30" s="65" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L30" s="153" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M30" s="19"/>
       <c r="N30" s="19"/>
@@ -5556,13 +5445,13 @@
       <c r="I32" s="19"/>
       <c r="J32" s="21"/>
       <c r="K32" s="65" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="L32" s="64" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M32" s="153" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N32" s="19"/>
       <c r="O32" s="20"/>
@@ -5609,10 +5498,10 @@
       <c r="J34" s="21"/>
       <c r="K34" s="19"/>
       <c r="L34" s="64" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="M34" s="153" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N34" s="19"/>
       <c r="O34" s="20"/>
@@ -5663,7 +5552,7 @@
       <c r="H36" s="91"/>
       <c r="I36" s="91"/>
       <c r="J36" s="17"/>
-      <c r="K36" s="92"/>
+      <c r="K36" s="163"/>
       <c r="L36" s="91"/>
       <c r="M36" s="91"/>
       <c r="N36" s="91"/>
@@ -5685,18 +5574,12 @@
       <c r="E37" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I37" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="F37" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="G37" s="20"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
       <c r="J37" s="21"/>
       <c r="K37" s="20"/>
       <c r="L37" s="19"/>
@@ -5720,25 +5603,15 @@
       <c r="G38" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I38" s="23" t="s">
-        <v>34</v>
-      </c>
+      <c r="H38" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" s="19"/>
       <c r="J38" s="21"/>
-      <c r="K38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N38" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="K38" s="20"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+      <c r="N38" s="19"/>
       <c r="O38" s="20"/>
       <c r="P38" s="19"/>
       <c r="Q38" s="22"/>
@@ -5755,65 +5628,61 @@
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="20"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
+      <c r="H39" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="151" t="s">
+        <v>34</v>
+      </c>
       <c r="J39" s="21"/>
       <c r="K39" s="20"/>
       <c r="L39" s="19"/>
       <c r="M39" s="19"/>
       <c r="N39" s="19"/>
-      <c r="O39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="P39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q39" s="150" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="96" t="s">
+      <c r="O39" s="20"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="22"/>
+    </row>
+    <row r="40" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="94" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="97" t="s">
+      <c r="B40" s="95" t="s">
         <v>69</v>
       </c>
-      <c r="C40" s="158"/>
-      <c r="D40" s="98"/>
-      <c r="E40" s="98"/>
-      <c r="F40" s="98"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="98"/>
-      <c r="I40" s="98"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="99"/>
-      <c r="L40" s="98"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="98"/>
-      <c r="O40" s="99"/>
-      <c r="P40" s="98"/>
-      <c r="Q40" s="100" t="s">
-        <v>17</v>
-      </c>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N40" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O40" s="20"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="22"/>
     </row>
     <row r="41" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="101" t="s">
+      <c r="A41" s="94" t="s">
         <v>70</v>
       </c>
-      <c r="B41" s="102" t="s">
+      <c r="B41" s="95" t="s">
         <v>71</v>
       </c>
       <c r="C41" s="19"/>
-      <c r="D41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="159" t="s">
-        <v>20</v>
-      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
       <c r="G41" s="20"/>
       <c r="H41" s="19"/>
       <c r="I41" s="19"/>
@@ -5822,48 +5691,40 @@
       <c r="L41" s="19"/>
       <c r="M41" s="19"/>
       <c r="N41" s="19"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="19"/>
-      <c r="Q41" s="22"/>
-    </row>
-    <row r="42" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="101" t="s">
+      <c r="O41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="P41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q41" s="150" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="96" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="102" t="s">
+      <c r="B42" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="J42" s="21"/>
-      <c r="K42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N42" s="151" t="s">
-        <v>34</v>
-      </c>
-      <c r="O42" s="20"/>
-      <c r="P42" s="19"/>
-      <c r="Q42" s="22"/>
+      <c r="C42" s="158"/>
+      <c r="D42" s="98"/>
+      <c r="E42" s="98"/>
+      <c r="F42" s="98"/>
+      <c r="G42" s="99"/>
+      <c r="H42" s="98"/>
+      <c r="I42" s="98"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="99"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="98"/>
+      <c r="O42" s="99"/>
+      <c r="P42" s="98"/>
+      <c r="Q42" s="100" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="43" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="101" t="s">
@@ -5873,173 +5734,241 @@
         <v>75</v>
       </c>
       <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
+      <c r="D43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="159" t="s">
+        <v>20</v>
+      </c>
       <c r="G43" s="20"/>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
       <c r="J43" s="21"/>
       <c r="K43" s="20"/>
       <c r="L43" s="19"/>
-      <c r="M43" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N43" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
       <c r="O43" s="20"/>
       <c r="P43" s="19"/>
       <c r="Q43" s="22"/>
     </row>
     <row r="44" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="103" t="s">
+      <c r="A44" s="101" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="104" t="s">
+      <c r="B44" s="102" t="s">
         <v>77</v>
       </c>
-      <c r="C44" s="105"/>
-      <c r="D44" s="105"/>
-      <c r="E44" s="105"/>
-      <c r="F44" s="105"/>
-      <c r="G44" s="106"/>
-      <c r="H44" s="105"/>
-      <c r="I44" s="105"/>
-      <c r="J44" s="107"/>
-      <c r="K44" s="106"/>
-      <c r="L44" s="105"/>
-      <c r="M44" s="105"/>
-      <c r="N44" s="105"/>
-      <c r="O44" s="108" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="J44" s="21"/>
+      <c r="K44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="L44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N44" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O44" s="20"/>
+      <c r="P44" s="19"/>
+      <c r="Q44" s="22"/>
+    </row>
+    <row r="45" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="101" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="102" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="19"/>
+      <c r="I45" s="19"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N45" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O45" s="20"/>
+      <c r="P45" s="19"/>
+      <c r="Q45" s="22"/>
+    </row>
+    <row r="46" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="103" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="106"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="107"/>
+      <c r="K46" s="106"/>
+      <c r="L46" s="105"/>
+      <c r="M46" s="105"/>
+      <c r="N46" s="105"/>
+      <c r="O46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="P44" s="108" t="s">
+      <c r="P46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="150" t="s">
+      <c r="Q46" s="150" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="186" t="s">
-        <v>105</v>
-      </c>
-      <c r="B45" s="187"/>
-      <c r="C45" s="187"/>
-      <c r="D45" s="187"/>
-      <c r="E45" s="187"/>
-      <c r="F45" s="187"/>
-      <c r="G45" s="187"/>
-      <c r="H45" s="187"/>
-      <c r="I45" s="187"/>
-      <c r="J45" s="187"/>
-      <c r="K45" s="187"/>
-      <c r="L45" s="187"/>
-      <c r="M45" s="187"/>
-      <c r="N45" s="187"/>
-      <c r="O45" s="187"/>
-      <c r="P45" s="187"/>
-      <c r="Q45" s="187"/>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C46" s="109" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="110" t="s">
-        <v>80</v>
-      </c>
-      <c r="D47" s="167" t="s">
-        <v>81</v>
-      </c>
-      <c r="E47" s="168"/>
-    </row>
-    <row r="48" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="111" t="s">
+    <row r="47" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="187" t="s">
+        <v>109</v>
+      </c>
+      <c r="B47" s="188"/>
+      <c r="C47" s="188"/>
+      <c r="D47" s="188"/>
+      <c r="E47" s="188"/>
+      <c r="F47" s="188"/>
+      <c r="G47" s="188"/>
+      <c r="H47" s="188"/>
+      <c r="I47" s="188"/>
+      <c r="J47" s="188"/>
+      <c r="K47" s="188"/>
+      <c r="L47" s="188"/>
+      <c r="M47" s="188"/>
+      <c r="N47" s="188"/>
+      <c r="O47" s="188"/>
+      <c r="P47" s="188"/>
+      <c r="Q47" s="188"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C48" s="109" t="s">
         <v>83</v>
       </c>
-      <c r="D48" s="169" t="s">
+    </row>
+    <row r="49" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C49" s="110" t="s">
         <v>84</v>
       </c>
-      <c r="E48" s="170"/>
-    </row>
-    <row r="49" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="112" t="s">
-        <v>86</v>
-      </c>
-      <c r="D49" s="181" t="s">
+      <c r="D49" s="176" t="s">
+        <v>85</v>
+      </c>
+      <c r="E49" s="177"/>
+    </row>
+    <row r="50" spans="3:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="E49" s="182"/>
+      <c r="D50" s="182" t="s">
+        <v>88</v>
+      </c>
+      <c r="E50" s="183"/>
     </row>
     <row r="51" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="113" t="s">
-        <v>89</v>
-      </c>
-      <c r="D51" s="114" t="s">
+      <c r="C51" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="F51" s="114" t="s">
+      <c r="D51" s="172" t="s">
         <v>91</v>
       </c>
-      <c r="H51" s="114" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="52" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D52" s="114" t="s">
+      <c r="E51" s="173"/>
+    </row>
+    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="113" t="s">
         <v>93</v>
       </c>
-      <c r="F52" s="114" t="s">
+      <c r="D53" s="114" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D53" s="114" t="s">
+      <c r="F53" s="114" t="s">
         <v>95</v>
       </c>
-      <c r="F53" s="114"/>
+      <c r="H53" s="114" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="54" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="113" t="s">
-        <v>96</v>
-      </c>
       <c r="D54" s="114" t="s">
         <v>97</v>
       </c>
-      <c r="E54" s="114" t="s">
+      <c r="F54" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="F54" s="114" t="s">
+    </row>
+    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D55" s="114" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="113" t="s">
+      <c r="F55" s="114"/>
+    </row>
+    <row r="56" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="113" t="s">
         <v>100</v>
       </c>
-      <c r="D55" s="151"/>
-      <c r="E55" s="149" t="s">
+      <c r="D56" s="114" t="s">
         <v>101</v>
+      </c>
+      <c r="E56" s="114" t="s">
+        <v>102</v>
+      </c>
+      <c r="F56" s="114" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="113" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" s="151"/>
+      <c r="E57" s="149" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="D47:E47"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="O1:Q1"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="O7:Q7"/>
     <mergeCell ref="K7:N7"/>
-    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D50:E50"/>
     <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="A45:Q45"/>
+    <mergeCell ref="A47:Q47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>
@@ -6051,7 +5980,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q55"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" customWidth="1"/>
@@ -6060,25 +5989,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O1" s="165" t="s">
+      <c r="O1" s="166" t="s">
         <v>0</v>
       </c>
-      <c r="P1" s="166"/>
-      <c r="Q1" s="166"/>
+      <c r="P1" s="167"/>
+      <c r="Q1" s="167"/>
     </row>
     <row r="2" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="O2" s="185" t="s">
+      <c r="O2" s="186" t="s">
         <v>2</v>
       </c>
-      <c r="P2" s="166"/>
-      <c r="Q2" s="166"/>
+      <c r="P2" s="167"/>
+      <c r="Q2" s="167"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:17" ht="4.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6103,43 +6032,43 @@
     <row r="5" spans="1:17" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="6" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="171" t="s">
+      <c r="A7" s="168" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="172"/>
-      <c r="C7" s="177" t="s">
+      <c r="B7" s="169"/>
+      <c r="C7" s="178" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="172"/>
-      <c r="E7" s="172"/>
-      <c r="F7" s="172"/>
-      <c r="G7" s="177" t="s">
+      <c r="D7" s="169"/>
+      <c r="E7" s="169"/>
+      <c r="F7" s="169"/>
+      <c r="G7" s="178" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="172"/>
-      <c r="I7" s="172"/>
-      <c r="J7" s="172"/>
-      <c r="K7" s="177" t="s">
+      <c r="H7" s="169"/>
+      <c r="I7" s="169"/>
+      <c r="J7" s="169"/>
+      <c r="K7" s="178" t="s">
         <v>8</v>
       </c>
-      <c r="L7" s="172"/>
-      <c r="M7" s="172"/>
-      <c r="N7" s="172"/>
-      <c r="O7" s="179" t="s">
+      <c r="L7" s="169"/>
+      <c r="M7" s="169"/>
+      <c r="N7" s="169"/>
+      <c r="O7" s="180" t="s">
         <v>9</v>
       </c>
-      <c r="P7" s="172"/>
-      <c r="Q7" s="180"/>
+      <c r="P7" s="169"/>
+      <c r="Q7" s="181"/>
     </row>
     <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="173" t="s">
+      <c r="A8" s="164" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="178" t="s">
+      <c r="B8" s="179" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="5">
@@ -6189,8 +6118,8 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="174"/>
-      <c r="B9" s="166"/>
+      <c r="A9" s="165"/>
+      <c r="B9" s="167"/>
       <c r="C9" s="11" t="s">
         <v>12</v>
       </c>
@@ -6545,13 +6474,13 @@
       <c r="B21" s="63"/>
       <c r="C21" s="19"/>
       <c r="D21" s="64" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E21" s="64" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F21" s="153" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G21" s="20"/>
       <c r="H21" s="19"/>
@@ -6578,10 +6507,12 @@
       <c r="F22" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="H22" s="19"/>
+      <c r="G22" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="I22" s="19"/>
       <c r="J22" s="21"/>
       <c r="K22" s="20"/>
@@ -6599,12 +6530,14 @@
       <c r="D23" s="19"/>
       <c r="E23" s="19"/>
       <c r="F23" s="64" t="s">
-        <v>108</v>
-      </c>
-      <c r="G23" s="153" t="s">
-        <v>108</v>
-      </c>
-      <c r="H23" s="19"/>
+        <v>112</v>
+      </c>
+      <c r="G23" s="64" t="s">
+        <v>112</v>
+      </c>
+      <c r="H23" s="153" t="s">
+        <v>112</v>
+      </c>
       <c r="I23" s="19"/>
       <c r="J23" s="21"/>
       <c r="K23" s="20"/>
@@ -6629,10 +6562,12 @@
       <c r="G24" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H24" s="152" t="s">
-        <v>34</v>
-      </c>
-      <c r="I24" s="19"/>
+      <c r="H24" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I24" s="152" t="s">
+        <v>34</v>
+      </c>
       <c r="J24" s="21"/>
       <c r="K24" s="20"/>
       <c r="L24" s="19"/>
@@ -6650,12 +6585,14 @@
       <c r="E25" s="19"/>
       <c r="F25" s="19"/>
       <c r="G25" s="65" t="s">
-        <v>108</v>
-      </c>
-      <c r="H25" s="153" t="s">
-        <v>108</v>
-      </c>
-      <c r="I25" s="19"/>
+        <v>112</v>
+      </c>
+      <c r="H25" s="65" t="s">
+        <v>112</v>
+      </c>
+      <c r="I25" s="153" t="s">
+        <v>112</v>
+      </c>
       <c r="J25" s="21"/>
       <c r="K25" s="20"/>
       <c r="L25" s="19"/>
@@ -6781,10 +6718,10 @@
       <c r="I30" s="19"/>
       <c r="J30" s="21"/>
       <c r="K30" s="65" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="L30" s="153" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="M30" s="19"/>
       <c r="N30" s="19"/>
@@ -6833,13 +6770,13 @@
       <c r="I32" s="19"/>
       <c r="J32" s="21"/>
       <c r="K32" s="65" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="L32" s="64" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="M32" s="153" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N32" s="19"/>
       <c r="O32" s="20"/>
@@ -6886,10 +6823,10 @@
       <c r="J34" s="21"/>
       <c r="K34" s="19"/>
       <c r="L34" s="64" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="M34" s="153" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="N34" s="19"/>
       <c r="O34" s="20"/>
@@ -6940,7 +6877,7 @@
       <c r="H36" s="91"/>
       <c r="I36" s="91"/>
       <c r="J36" s="17"/>
-      <c r="K36" s="92"/>
+      <c r="K36" s="163"/>
       <c r="L36" s="91"/>
       <c r="M36" s="91"/>
       <c r="N36" s="91"/>
@@ -6962,18 +6899,12 @@
       <c r="E37" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="F37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H37" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I37" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="F37" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="G37" s="20"/>
+      <c r="H37" s="19"/>
+      <c r="I37" s="19"/>
       <c r="J37" s="21"/>
       <c r="K37" s="20"/>
       <c r="L37" s="19"/>
@@ -6997,25 +6928,15 @@
       <c r="G38" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I38" s="23" t="s">
-        <v>34</v>
-      </c>
+      <c r="H38" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="I38" s="19"/>
       <c r="J38" s="21"/>
-      <c r="K38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M38" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N38" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="K38" s="20"/>
+      <c r="L38" s="19"/>
+      <c r="M38" s="19"/>
+      <c r="N38" s="19"/>
       <c r="O38" s="20"/>
       <c r="P38" s="19"/>
       <c r="Q38" s="22"/>
@@ -7032,65 +6953,61 @@
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="20"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
+      <c r="H39" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I39" s="151" t="s">
+        <v>34</v>
+      </c>
       <c r="J39" s="21"/>
       <c r="K39" s="20"/>
       <c r="L39" s="19"/>
       <c r="M39" s="19"/>
       <c r="N39" s="19"/>
-      <c r="O39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="P39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q39" s="150" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="40" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="96" t="s">
+      <c r="O39" s="20"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="22"/>
+    </row>
+    <row r="40" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="94" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="97" t="s">
+      <c r="B40" s="95" t="s">
         <v>69</v>
       </c>
-      <c r="C40" s="158"/>
-      <c r="D40" s="98"/>
-      <c r="E40" s="98"/>
-      <c r="F40" s="98"/>
-      <c r="G40" s="99"/>
-      <c r="H40" s="98"/>
-      <c r="I40" s="98"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="99"/>
-      <c r="L40" s="98"/>
-      <c r="M40" s="98"/>
-      <c r="N40" s="98"/>
-      <c r="O40" s="99"/>
-      <c r="P40" s="98"/>
-      <c r="Q40" s="100" t="s">
-        <v>17</v>
-      </c>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="20"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="20"/>
+      <c r="L40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M40" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N40" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O40" s="20"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="22"/>
     </row>
     <row r="41" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="101" t="s">
+      <c r="A41" s="94" t="s">
         <v>70</v>
       </c>
-      <c r="B41" s="102" t="s">
+      <c r="B41" s="95" t="s">
         <v>71</v>
       </c>
       <c r="C41" s="19"/>
-      <c r="D41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E41" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="159" t="s">
-        <v>20</v>
-      </c>
+      <c r="D41" s="19"/>
+      <c r="E41" s="19"/>
+      <c r="F41" s="19"/>
       <c r="G41" s="20"/>
       <c r="H41" s="19"/>
       <c r="I41" s="19"/>
@@ -7099,48 +7016,40 @@
       <c r="L41" s="19"/>
       <c r="M41" s="19"/>
       <c r="N41" s="19"/>
-      <c r="O41" s="20"/>
-      <c r="P41" s="19"/>
-      <c r="Q41" s="22"/>
-    </row>
-    <row r="42" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="101" t="s">
+      <c r="O41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="P41" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q41" s="150" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="26.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="96" t="s">
         <v>72</v>
       </c>
-      <c r="B42" s="102" t="s">
+      <c r="B42" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="C42" s="19"/>
-      <c r="D42" s="19"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="G42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="I42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="J42" s="21"/>
-      <c r="K42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="L42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="M42" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N42" s="151" t="s">
-        <v>34</v>
-      </c>
-      <c r="O42" s="20"/>
-      <c r="P42" s="19"/>
-      <c r="Q42" s="22"/>
+      <c r="C42" s="158"/>
+      <c r="D42" s="98"/>
+      <c r="E42" s="98"/>
+      <c r="F42" s="98"/>
+      <c r="G42" s="99"/>
+      <c r="H42" s="98"/>
+      <c r="I42" s="98"/>
+      <c r="J42" s="17"/>
+      <c r="K42" s="99"/>
+      <c r="L42" s="98"/>
+      <c r="M42" s="98"/>
+      <c r="N42" s="98"/>
+      <c r="O42" s="99"/>
+      <c r="P42" s="98"/>
+      <c r="Q42" s="100" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="43" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="101" t="s">
@@ -7150,173 +7059,241 @@
         <v>75</v>
       </c>
       <c r="C43" s="19"/>
-      <c r="D43" s="19"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="19"/>
+      <c r="D43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="E43" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="159" t="s">
+        <v>20</v>
+      </c>
       <c r="G43" s="20"/>
       <c r="H43" s="19"/>
       <c r="I43" s="19"/>
       <c r="J43" s="21"/>
       <c r="K43" s="20"/>
       <c r="L43" s="19"/>
-      <c r="M43" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="N43" s="151" t="s">
-        <v>34</v>
-      </c>
+      <c r="M43" s="19"/>
+      <c r="N43" s="19"/>
       <c r="O43" s="20"/>
       <c r="P43" s="19"/>
       <c r="Q43" s="22"/>
     </row>
     <row r="44" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="103" t="s">
+      <c r="A44" s="101" t="s">
         <v>76</v>
       </c>
-      <c r="B44" s="104" t="s">
+      <c r="B44" s="102" t="s">
         <v>77</v>
       </c>
-      <c r="C44" s="105"/>
-      <c r="D44" s="105"/>
-      <c r="E44" s="105"/>
-      <c r="F44" s="105"/>
-      <c r="G44" s="106"/>
-      <c r="H44" s="105"/>
-      <c r="I44" s="105"/>
-      <c r="J44" s="107"/>
-      <c r="K44" s="106"/>
-      <c r="L44" s="105"/>
-      <c r="M44" s="105"/>
-      <c r="N44" s="105"/>
-      <c r="O44" s="108" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="19"/>
+      <c r="F44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="H44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="I44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="J44" s="21"/>
+      <c r="K44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="L44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="M44" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N44" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O44" s="20"/>
+      <c r="P44" s="19"/>
+      <c r="Q44" s="22"/>
+    </row>
+    <row r="45" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="101" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="102" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="19"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="19"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="20"/>
+      <c r="H45" s="19"/>
+      <c r="I45" s="19"/>
+      <c r="J45" s="21"/>
+      <c r="K45" s="20"/>
+      <c r="L45" s="19"/>
+      <c r="M45" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="N45" s="151" t="s">
+        <v>34</v>
+      </c>
+      <c r="O45" s="20"/>
+      <c r="P45" s="19"/>
+      <c r="Q45" s="22"/>
+    </row>
+    <row r="46" spans="1:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="103" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="104" t="s">
+        <v>81</v>
+      </c>
+      <c r="C46" s="105"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="105"/>
+      <c r="F46" s="105"/>
+      <c r="G46" s="106"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="105"/>
+      <c r="J46" s="107"/>
+      <c r="K46" s="106"/>
+      <c r="L46" s="105"/>
+      <c r="M46" s="105"/>
+      <c r="N46" s="105"/>
+      <c r="O46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="P44" s="108" t="s">
+      <c r="P46" s="108" t="s">
         <v>20</v>
       </c>
-      <c r="Q44" s="150" t="s">
+      <c r="Q46" s="150" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="186" t="s">
-        <v>109</v>
-      </c>
-      <c r="B45" s="187"/>
-      <c r="C45" s="187"/>
-      <c r="D45" s="187"/>
-      <c r="E45" s="187"/>
-      <c r="F45" s="187"/>
-      <c r="G45" s="187"/>
-      <c r="H45" s="187"/>
-      <c r="I45" s="187"/>
-      <c r="J45" s="187"/>
-      <c r="K45" s="187"/>
-      <c r="L45" s="187"/>
-      <c r="M45" s="187"/>
-      <c r="N45" s="187"/>
-      <c r="O45" s="187"/>
-      <c r="P45" s="187"/>
-      <c r="Q45" s="187"/>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="C46" s="109" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="47" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="110" t="s">
-        <v>80</v>
-      </c>
-      <c r="D47" s="167" t="s">
-        <v>82</v>
-      </c>
-      <c r="E47" s="168"/>
-    </row>
-    <row r="48" spans="1:17" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C48" s="111" t="s">
+    <row r="47" spans="1:17" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="187" t="s">
+        <v>113</v>
+      </c>
+      <c r="B47" s="188"/>
+      <c r="C47" s="188"/>
+      <c r="D47" s="188"/>
+      <c r="E47" s="188"/>
+      <c r="F47" s="188"/>
+      <c r="G47" s="188"/>
+      <c r="H47" s="188"/>
+      <c r="I47" s="188"/>
+      <c r="J47" s="188"/>
+      <c r="K47" s="188"/>
+      <c r="L47" s="188"/>
+      <c r="M47" s="188"/>
+      <c r="N47" s="188"/>
+      <c r="O47" s="188"/>
+      <c r="P47" s="188"/>
+      <c r="Q47" s="188"/>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="C48" s="109" t="s">
         <v>83</v>
       </c>
-      <c r="D48" s="169" t="s">
-        <v>85</v>
-      </c>
-      <c r="E48" s="170"/>
     </row>
     <row r="49" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="112" t="s">
+      <c r="C49" s="110" t="s">
+        <v>84</v>
+      </c>
+      <c r="D49" s="176" t="s">
         <v>86</v>
       </c>
-      <c r="D49" s="181" t="s">
-        <v>88</v>
-      </c>
-      <c r="E49" s="182"/>
+      <c r="E49" s="177"/>
+    </row>
+    <row r="50" spans="3:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C50" s="111" t="s">
+        <v>87</v>
+      </c>
+      <c r="D50" s="182" t="s">
+        <v>89</v>
+      </c>
+      <c r="E50" s="183"/>
     </row>
     <row r="51" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C51" s="113" t="s">
-        <v>89</v>
-      </c>
-      <c r="D51" s="114" t="s">
+      <c r="C51" s="112" t="s">
         <v>90</v>
       </c>
-      <c r="F51" s="114" t="s">
-        <v>91</v>
-      </c>
-      <c r="H51" s="114" t="s">
+      <c r="D51" s="172" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="52" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D52" s="114" t="s">
+      <c r="E51" s="173"/>
+    </row>
+    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C53" s="113" t="s">
         <v>93</v>
       </c>
-      <c r="F52" s="114" t="s">
+      <c r="D53" s="114" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="53" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D53" s="114" t="s">
+      <c r="F53" s="114" t="s">
         <v>95</v>
       </c>
-      <c r="F53" s="114"/>
+      <c r="H53" s="114" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="54" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="113" t="s">
-        <v>96</v>
-      </c>
       <c r="D54" s="114" t="s">
         <v>97</v>
       </c>
-      <c r="E54" s="114" t="s">
+      <c r="F54" s="114" t="s">
         <v>98</v>
       </c>
-      <c r="F54" s="114" t="s">
+    </row>
+    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D55" s="114" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="55" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="113" t="s">
+      <c r="F55" s="114"/>
+    </row>
+    <row r="56" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C56" s="113" t="s">
         <v>100</v>
       </c>
-      <c r="D55" s="151"/>
-      <c r="E55" s="149" t="s">
+      <c r="D56" s="114" t="s">
         <v>101</v>
+      </c>
+      <c r="E56" s="114" t="s">
+        <v>102</v>
+      </c>
+      <c r="F56" s="114" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="57" spans="3:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C57" s="113" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" s="151"/>
+      <c r="E57" s="149" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="D47:E47"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="O1:Q1"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D51:E51"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="O7:Q7"/>
     <mergeCell ref="K7:N7"/>
-    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D50:E50"/>
     <mergeCell ref="O2:Q2"/>
-    <mergeCell ref="A45:Q45"/>
+    <mergeCell ref="A47:Q47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="8" fitToHeight="0" orientation="landscape"/>
@@ -7328,7 +7305,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -7340,12 +7317,12 @@
   <sheetData>
     <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="113" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -7353,26 +7330,26 @@
         <v>10</v>
       </c>
       <c r="B4" s="115" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C4" s="115" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D4" s="115" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="E4" s="115" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="196" t="s">
-        <v>116</v>
-      </c>
-      <c r="B5" s="197"/>
-      <c r="C5" s="197"/>
-      <c r="D5" s="197"/>
-      <c r="E5" s="197"/>
+      <c r="A5" s="195" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="196"/>
+      <c r="C5" s="196"/>
+      <c r="D5" s="196"/>
+      <c r="E5" s="196"/>
     </row>
     <row r="6" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="120" t="s">
@@ -7382,7 +7359,7 @@
         <v>19</v>
       </c>
       <c r="C6" s="117" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D6" s="118">
         <v>2</v>
@@ -7399,7 +7376,7 @@
         <v>22</v>
       </c>
       <c r="C7" s="117" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D7" s="118">
         <v>3</v>
@@ -7416,7 +7393,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="117" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D8" s="118">
         <v>5</v>
@@ -7433,7 +7410,7 @@
         <v>27</v>
       </c>
       <c r="C9" s="123" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D9" s="124">
         <v>4</v>
@@ -7443,13 +7420,13 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="190" t="s">
-        <v>121</v>
-      </c>
-      <c r="B10" s="191"/>
-      <c r="C10" s="191"/>
-      <c r="D10" s="191"/>
-      <c r="E10" s="191"/>
+      <c r="A10" s="189" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10" s="190"/>
+      <c r="C10" s="190"/>
+      <c r="D10" s="190"/>
+      <c r="E10" s="190"/>
     </row>
     <row r="11" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="126" t="s">
@@ -7459,7 +7436,7 @@
         <v>31</v>
       </c>
       <c r="C11" s="117" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D11" s="118">
         <v>1</v>
@@ -7476,7 +7453,7 @@
         <v>33</v>
       </c>
       <c r="C12" s="117" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D12" s="118">
         <v>2</v>
@@ -7493,7 +7470,7 @@
         <v>36</v>
       </c>
       <c r="C13" s="129" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D13" s="130">
         <v>2</v>
@@ -7503,13 +7480,13 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="198" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="199"/>
-      <c r="C14" s="199"/>
-      <c r="D14" s="199"/>
-      <c r="E14" s="199"/>
+      <c r="A14" s="197" t="s">
+        <v>127</v>
+      </c>
+      <c r="B14" s="198"/>
+      <c r="C14" s="198"/>
+      <c r="D14" s="198"/>
+      <c r="E14" s="198"/>
     </row>
     <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="131" t="s">
@@ -7519,13 +7496,13 @@
         <v>40</v>
       </c>
       <c r="C15" s="117" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D15" s="118">
         <v>3</v>
       </c>
       <c r="E15" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7536,13 +7513,13 @@
         <v>43</v>
       </c>
       <c r="C16" s="117" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D16" s="118">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7553,13 +7530,13 @@
         <v>45</v>
       </c>
       <c r="C17" s="117" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D17" s="118">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7570,7 +7547,7 @@
         <v>47</v>
       </c>
       <c r="C18" s="135" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D18" s="136">
         <v>1</v>
@@ -7580,13 +7557,13 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="194" t="s">
-        <v>128</v>
-      </c>
-      <c r="B19" s="195"/>
-      <c r="C19" s="195"/>
-      <c r="D19" s="195"/>
-      <c r="E19" s="195"/>
+      <c r="A19" s="193" t="s">
+        <v>132</v>
+      </c>
+      <c r="B19" s="194"/>
+      <c r="C19" s="194"/>
+      <c r="D19" s="194"/>
+      <c r="E19" s="194"/>
     </row>
     <row r="20" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="137" t="s">
@@ -7596,7 +7573,7 @@
         <v>51</v>
       </c>
       <c r="C20" s="117" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="D20" s="118">
         <v>2</v>
@@ -7613,13 +7590,13 @@
         <v>53</v>
       </c>
       <c r="C21" s="117" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D21" s="118">
         <v>2</v>
       </c>
       <c r="E21" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7630,13 +7607,13 @@
         <v>55</v>
       </c>
       <c r="C22" s="117" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D22" s="118">
         <v>3</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -7647,13 +7624,13 @@
         <v>57</v>
       </c>
       <c r="C23" s="117" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D23" s="118">
         <v>2</v>
       </c>
       <c r="E23" s="132" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -7664,7 +7641,7 @@
         <v>59</v>
       </c>
       <c r="C24" s="140" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D24" s="141">
         <v>3</v>
@@ -7674,13 +7651,13 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="192" t="s">
-        <v>134</v>
-      </c>
-      <c r="B25" s="193"/>
-      <c r="C25" s="193"/>
-      <c r="D25" s="193"/>
-      <c r="E25" s="193"/>
+      <c r="A25" s="191" t="s">
+        <v>138</v>
+      </c>
+      <c r="B25" s="192"/>
+      <c r="C25" s="192"/>
+      <c r="D25" s="192"/>
+      <c r="E25" s="192"/>
     </row>
     <row r="26" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="142" t="s">
@@ -7690,10 +7667,10 @@
         <v>63</v>
       </c>
       <c r="C26" s="117" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D26" s="118">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E26" s="23" t="s">
         <v>34</v>
@@ -7707,10 +7684,10 @@
         <v>65</v>
       </c>
       <c r="C27" s="117" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D27" s="118">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E27" s="23" t="s">
         <v>34</v>
@@ -7724,33 +7701,41 @@
         <v>67</v>
       </c>
       <c r="C28" s="117" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D28" s="118">
+        <v>2</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="142" t="s">
+        <v>68</v>
+      </c>
+      <c r="B29" s="116" t="s">
+        <v>69</v>
+      </c>
+      <c r="C29" s="117" t="s">
+        <v>141</v>
+      </c>
+      <c r="D29" s="118">
         <v>3</v>
       </c>
-      <c r="E28" s="24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="188" t="s">
-        <v>138</v>
-      </c>
-      <c r="B29" s="189"/>
-      <c r="C29" s="189"/>
-      <c r="D29" s="189"/>
-      <c r="E29" s="189"/>
+      <c r="E29" s="23" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="30" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="143" t="s">
+      <c r="A30" s="142" t="s">
         <v>70</v>
       </c>
       <c r="B30" s="116" t="s">
         <v>71</v>
       </c>
       <c r="C30" s="117" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="D30" s="118">
         <v>3</v>
@@ -7759,22 +7744,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="143" t="s">
-        <v>72</v>
-      </c>
-      <c r="B31" s="116" t="s">
-        <v>73</v>
-      </c>
-      <c r="C31" s="117" t="s">
-        <v>139</v>
-      </c>
-      <c r="D31" s="118">
-        <v>8</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>34</v>
-      </c>
+    <row r="31" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="199" t="s">
+        <v>143</v>
+      </c>
+      <c r="B31" s="200"/>
+      <c r="C31" s="200"/>
+      <c r="D31" s="200"/>
+      <c r="E31" s="200"/>
     </row>
     <row r="32" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="143" t="s">
@@ -7784,35 +7761,69 @@
         <v>75</v>
       </c>
       <c r="C32" s="117" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="D32" s="118">
+        <v>3</v>
+      </c>
+      <c r="E32" s="24" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="143" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="116" t="s">
+        <v>77</v>
+      </c>
+      <c r="C33" s="117" t="s">
+        <v>144</v>
+      </c>
+      <c r="D33" s="118">
+        <v>8</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="143" t="s">
+        <v>78</v>
+      </c>
+      <c r="B34" s="116" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" s="117" t="s">
+        <v>145</v>
+      </c>
+      <c r="D34" s="118">
         <v>2</v>
       </c>
-      <c r="E32" s="23" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="144" t="s">
-        <v>76</v>
-      </c>
-      <c r="B33" s="145" t="s">
-        <v>77</v>
-      </c>
-      <c r="C33" s="146" t="s">
-        <v>137</v>
-      </c>
-      <c r="D33" s="147">
+      <c r="E34" s="23" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="144" t="s">
+        <v>80</v>
+      </c>
+      <c r="B35" s="145" t="s">
+        <v>81</v>
+      </c>
+      <c r="C35" s="146" t="s">
+        <v>142</v>
+      </c>
+      <c r="D35" s="147">
         <v>3</v>
       </c>
-      <c r="E33" s="24" t="s">
+      <c r="E35" s="24" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A10:E10"/>
     <mergeCell ref="A25:E25"/>
     <mergeCell ref="A19:E19"/>

</xml_diff>